<commit_message>
Compilation error fix. move to spring ai 1.0.0
</commit_message>
<xml_diff>
--- a/src/main/resources/about/jsonplaceholder_user_details.xlsx
+++ b/src/main/resources/about/jsonplaceholder_user_details.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t xml:space="preserve">Bret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not available</t>
   </si>
   <si>
     <r>
@@ -42,6 +45,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Meet Bret! Bret, whose real name is </t>
     </r>
@@ -51,6 +55,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Leanne Graham</t>
     </r>
@@ -59,6 +64,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">, is a dynamic professional with a knack for technology and business innovation. He is associated with Romaguera-Crona, a forward-thinking company known for its expertise in multi-layered client-server neural networks. Bret plays a role in harnessing real-time e-markets, ensuring efficiency and adaptability in the digital landscape.
 Residing in Gwenborough, he enjoys the suburban comfort of Kulas Light, Apt. 556. His communication game is strong—whether it’s via email at Sincere@april.biz or through his phone at 1-770-736-8031 x56442. When he’s not immersed in work, he might be found browsing his company’s website, hildegard.org, for the latest developments.
@@ -79,6 +85,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -100,6 +107,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -149,11 +157,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -167,48 +175,6 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>465840</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>39240</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr=""/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1625760" y="162720"/>
-          <a:ext cx="2904120" cy="4202640"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -325,7 +291,9 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="29.77"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -342,15 +310,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="1053.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -361,6 +332,5 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>